<commit_message>
Add Technician Solved Pivot Matrix table to dashboard and Excel reports
</commit_message>
<xml_diff>
--- a/EXECUTIVE_TEAM_AUDIT_REPORT_14_Sep_2026.xlsx
+++ b/EXECUTIVE_TEAM_AUDIT_REPORT_14_Sep_2026.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet name="Team Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Category Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Master Audit Details" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Technician Matrix Pivot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Master Audit Details" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,8 +44,14 @@
       <color rgb="001F4E78"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -61,6 +68,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
         <bgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -90,13 +103,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -747,7 +761,297 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX45"/>
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sub Category</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Chandramani Tharu</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Rajesh Maharjan</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Sabin Giri</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Sanjeev Giri</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Shashikant Chaudhary</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Sunil Chaudhary</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Grand Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Router Upgrade  Wi-Fi 6</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="H2" s="4" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Router Adaptor damage Issue</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>IPTV STB box Damage Issue</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>NETTV-Channel buffering,feeze issue</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Router Damage Issue</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Specific Website/App is slow</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Video content is Buffering</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Grand Total</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AY45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -800,6 +1104,7 @@
     <col width="45" customWidth="1" min="48" max="48"/>
     <col width="25" customWidth="1" min="49" max="49"/>
     <col width="23" customWidth="1" min="50" max="50"/>
+    <col width="16" customWidth="1" min="51" max="51"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1053,6 +1358,11 @@
           <t>Employee Name</t>
         </is>
       </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>Is_Solved_Val</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1121,10 +1431,8 @@
           <t>Bhanu Pandit</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>9851048677</t>
-        </is>
+      <c r="O2" s="2" t="n">
+        <v>9851048677</v>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
@@ -1159,10 +1467,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y2" s="2" t="inlineStr">
-        <is>
-          <t>27.65686</t>
-        </is>
+      <c r="Y2" s="2" t="n">
+        <v>27.65686</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1218,20 +1524,16 @@
           <t>Rajesh Maharjan</t>
         </is>
       </c>
-      <c r="AN2" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="AN2" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="AO2" s="2" t="inlineStr">
         <is>
           <t>3,10</t>
         </is>
       </c>
-      <c r="AP2" s="2" t="inlineStr">
-        <is>
-          <t>85.30276</t>
-        </is>
+      <c r="AP2" s="2" t="n">
+        <v>85.30276000000001</v>
       </c>
       <c r="AQ2" s="2" t="inlineStr"/>
       <c r="AR2" s="2" t="inlineStr">
@@ -1268,6 +1570,9 @@
         <is>
           <t>Rajesh Maharjan</t>
         </is>
+      </c>
+      <c r="AY2" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -1337,10 +1642,8 @@
           <t>Surakshya Thapa Magar</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>9746488661</t>
-        </is>
+      <c r="O3" s="2" t="n">
+        <v>9746488661</v>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
@@ -1375,10 +1678,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y3" s="2" t="inlineStr">
-        <is>
-          <t>27.658596</t>
-        </is>
+      <c r="Y3" s="2" t="n">
+        <v>27.658596</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1430,20 +1731,16 @@
           <t>Rajesh Maharjan</t>
         </is>
       </c>
-      <c r="AN3" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN3" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO3" s="2" t="inlineStr">
         <is>
           <t>CDB202</t>
         </is>
       </c>
-      <c r="AP3" s="2" t="inlineStr">
-        <is>
-          <t>85.31129</t>
-        </is>
+      <c r="AP3" s="2" t="n">
+        <v>85.31129</v>
       </c>
       <c r="AQ3" s="2" t="inlineStr"/>
       <c r="AR3" s="2" t="inlineStr">
@@ -1480,6 +1777,9 @@
         <is>
           <t>Rajesh Maharjan</t>
         </is>
+      </c>
+      <c r="AY3" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -1549,10 +1849,8 @@
           <t>Raju Maharjan</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>9843910198</t>
-        </is>
+      <c r="O4" s="2" t="n">
+        <v>9843910198</v>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
@@ -1587,10 +1885,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y4" s="2" t="inlineStr">
-        <is>
-          <t>27.68274</t>
-        </is>
+      <c r="Y4" s="2" t="n">
+        <v>27.68274</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1646,20 +1942,16 @@
           <t>Rajesh Maharjan</t>
         </is>
       </c>
-      <c r="AN4" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="AN4" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="AO4" s="2" t="inlineStr">
         <is>
           <t>3,2</t>
         </is>
       </c>
-      <c r="AP4" s="2" t="inlineStr">
-        <is>
-          <t>85.27882</t>
-        </is>
+      <c r="AP4" s="2" t="n">
+        <v>85.27882</v>
       </c>
       <c r="AQ4" s="2" t="inlineStr"/>
       <c r="AR4" s="2" t="inlineStr">
@@ -1696,6 +1988,9 @@
         <is>
           <t>Rajesh Maharjan</t>
         </is>
+      </c>
+      <c r="AY4" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -1765,10 +2060,8 @@
           <t>Nirajan Regmi</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
-        <is>
-          <t>9861446023</t>
-        </is>
+      <c r="O5" s="2" t="n">
+        <v>9861446023</v>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
@@ -1803,10 +2096,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y5" s="2" t="inlineStr">
-        <is>
-          <t>27.661336</t>
-        </is>
+      <c r="Y5" s="2" t="n">
+        <v>27.661336</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1862,20 +2153,16 @@
           <t>Shashikant Chaudhary</t>
         </is>
       </c>
-      <c r="AN5" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="AN5" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="AO5" s="2" t="inlineStr">
         <is>
           <t>3,15</t>
         </is>
       </c>
-      <c r="AP5" s="2" t="inlineStr">
-        <is>
-          <t>85.37222</t>
-        </is>
+      <c r="AP5" s="2" t="n">
+        <v>85.37222</v>
       </c>
       <c r="AQ5" s="2" t="inlineStr"/>
       <c r="AR5" s="2" t="inlineStr">
@@ -1912,6 +2199,9 @@
         <is>
           <t>Shashikant Chaudhary</t>
         </is>
+      </c>
+      <c r="AY5" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -1981,10 +2271,8 @@
           <t>Suman Neupane</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>9844674481</t>
-        </is>
+      <c r="O6" s="2" t="n">
+        <v>9844674481</v>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
@@ -2019,10 +2307,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y6" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="Y6" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2078,20 +2364,16 @@
           <t>Shashikant Chaudhary</t>
         </is>
       </c>
-      <c r="AN6" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="AN6" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="AO6" s="2" t="inlineStr">
         <is>
           <t>3,16</t>
         </is>
       </c>
-      <c r="AP6" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="AP6" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="AQ6" s="2" t="inlineStr"/>
       <c r="AR6" s="2" t="inlineStr">
@@ -2128,6 +2410,9 @@
         <is>
           <t>Shashikant Chaudhary</t>
         </is>
+      </c>
+      <c r="AY6" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -2197,10 +2482,8 @@
           <t>Uma Khatri</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>9762419916</t>
-        </is>
+      <c r="O7" s="2" t="n">
+        <v>9762419916</v>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
@@ -2235,10 +2518,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y7" s="2" t="inlineStr">
-        <is>
-          <t>27.65472</t>
-        </is>
+      <c r="Y7" s="2" t="n">
+        <v>27.65472</v>
       </c>
       <c r="Z7" s="2" t="inlineStr">
         <is>
@@ -2294,20 +2575,16 @@
           <t>Rahul Chaudhary</t>
         </is>
       </c>
-      <c r="AN7" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="AN7" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="AO7" s="2" t="inlineStr">
         <is>
           <t>1,14</t>
         </is>
       </c>
-      <c r="AP7" s="2" t="inlineStr">
-        <is>
-          <t>85.33054</t>
-        </is>
+      <c r="AP7" s="2" t="n">
+        <v>85.33054</v>
       </c>
       <c r="AQ7" s="2" t="inlineStr"/>
       <c r="AR7" s="2" t="inlineStr">
@@ -2344,6 +2621,9 @@
         <is>
           <t>Shashikant Chaudhary</t>
         </is>
+      </c>
+      <c r="AY7" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -2413,10 +2693,8 @@
           <t>Menuka Bista</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>9841436927</t>
-        </is>
+      <c r="O8" s="2" t="n">
+        <v>9841436927</v>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
@@ -2506,10 +2784,8 @@
           <t>Binod Dhami</t>
         </is>
       </c>
-      <c r="AN8" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN8" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO8" s="2" t="inlineStr">
         <is>
@@ -2553,6 +2829,9 @@
           <t>Shashikant Chaudhary</t>
         </is>
       </c>
+      <c r="AY8" s="2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2621,10 +2900,8 @@
           <t>Girish Ojha</t>
         </is>
       </c>
-      <c r="O9" s="2" t="inlineStr">
-        <is>
-          <t>9823402588</t>
-        </is>
+      <c r="O9" s="2" t="n">
+        <v>9823402588</v>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
@@ -2659,10 +2936,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y9" s="2" t="inlineStr">
-        <is>
-          <t>27.67367</t>
-        </is>
+      <c r="Y9" s="2" t="n">
+        <v>27.67367</v>
       </c>
       <c r="Z9" s="2" t="inlineStr">
         <is>
@@ -2714,20 +2989,16 @@
           <t>Shashikant Chaudhary</t>
         </is>
       </c>
-      <c r="AN9" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="AN9" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="AO9" s="2" t="inlineStr">
         <is>
           <t>4,10</t>
         </is>
       </c>
-      <c r="AP9" s="2" t="inlineStr">
-        <is>
-          <t>85.35165</t>
-        </is>
+      <c r="AP9" s="2" t="n">
+        <v>85.35165000000001</v>
       </c>
       <c r="AQ9" s="2" t="inlineStr"/>
       <c r="AR9" s="2" t="inlineStr">
@@ -2764,6 +3035,9 @@
         <is>
           <t>Shashikant Chaudhary</t>
         </is>
+      </c>
+      <c r="AY9" s="2" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -2833,10 +3107,8 @@
           <t>Sangita Rai</t>
         </is>
       </c>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>9767945255</t>
-        </is>
+      <c r="O10" s="2" t="n">
+        <v>9767945255</v>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
@@ -2871,10 +3143,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y10" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="Y10" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="Z10" s="2" t="inlineStr">
         <is>
@@ -2930,20 +3200,16 @@
           <t>Sabin Giri</t>
         </is>
       </c>
-      <c r="AN10" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN10" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO10" s="2" t="inlineStr">
         <is>
           <t>L43-8</t>
         </is>
       </c>
-      <c r="AP10" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="AP10" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="AQ10" s="2" t="inlineStr"/>
       <c r="AR10" s="2" t="inlineStr">
@@ -2980,6 +3246,9 @@
         <is>
           <t>Sabin Giri</t>
         </is>
+      </c>
+      <c r="AY10" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -3049,10 +3318,8 @@
           <t>Bedika Dhungel</t>
         </is>
       </c>
-      <c r="O11" s="2" t="inlineStr">
-        <is>
-          <t>9820233663</t>
-        </is>
+      <c r="O11" s="2" t="n">
+        <v>9820233663</v>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
@@ -3087,10 +3354,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y11" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="Y11" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="Z11" s="2" t="inlineStr">
         <is>
@@ -3146,20 +3411,16 @@
           <t>Sabin Giri</t>
         </is>
       </c>
-      <c r="AN11" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN11" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO11" s="2" t="inlineStr">
         <is>
           <t>L57-4</t>
         </is>
       </c>
-      <c r="AP11" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="AP11" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="AQ11" s="2" t="inlineStr"/>
       <c r="AR11" s="2" t="inlineStr">
@@ -3196,6 +3457,9 @@
         <is>
           <t>Sabin Giri</t>
         </is>
+      </c>
+      <c r="AY11" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -3265,10 +3529,8 @@
           <t>Ashish nepal</t>
         </is>
       </c>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>9860326282</t>
-        </is>
+      <c r="O12" s="2" t="n">
+        <v>9860326282</v>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
@@ -3303,10 +3565,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y12" s="2" t="inlineStr">
-        <is>
-          <t>27.713806</t>
-        </is>
+      <c r="Y12" s="2" t="n">
+        <v>27.713806</v>
       </c>
       <c r="Z12" s="2" t="inlineStr">
         <is>
@@ -3362,20 +3622,16 @@
           <t>Sabin Giri</t>
         </is>
       </c>
-      <c r="AN12" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN12" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO12" s="2" t="inlineStr">
         <is>
           <t>L58-2</t>
         </is>
       </c>
-      <c r="AP12" s="2" t="inlineStr">
-        <is>
-          <t>85.357709</t>
-        </is>
+      <c r="AP12" s="2" t="n">
+        <v>85.357709</v>
       </c>
       <c r="AQ12" s="2" t="inlineStr"/>
       <c r="AR12" s="2" t="inlineStr">
@@ -3412,6 +3668,9 @@
         <is>
           <t>Sabin Giri</t>
         </is>
+      </c>
+      <c r="AY12" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -3481,10 +3740,8 @@
           <t>Prashant Shrestha</t>
         </is>
       </c>
-      <c r="O13" s="2" t="inlineStr">
-        <is>
-          <t>9813538454</t>
-        </is>
+      <c r="O13" s="2" t="n">
+        <v>9813538454</v>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
@@ -3519,10 +3776,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y13" s="2" t="inlineStr">
-        <is>
-          <t>27.76672</t>
-        </is>
+      <c r="Y13" s="2" t="n">
+        <v>27.76672</v>
       </c>
       <c r="Z13" s="2" t="inlineStr">
         <is>
@@ -3578,20 +3833,16 @@
           <t>Sabin Giri</t>
         </is>
       </c>
-      <c r="AN13" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN13" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO13" s="2" t="inlineStr">
         <is>
           <t>L44-7</t>
         </is>
       </c>
-      <c r="AP13" s="2" t="inlineStr">
-        <is>
-          <t>85.354</t>
-        </is>
+      <c r="AP13" s="2" t="n">
+        <v>85.354</v>
       </c>
       <c r="AQ13" s="2" t="inlineStr"/>
       <c r="AR13" s="2" t="inlineStr">
@@ -3628,6 +3879,9 @@
         <is>
           <t>Sabin Giri</t>
         </is>
+      </c>
+      <c r="AY13" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -3697,10 +3951,8 @@
           <t>Omprakash Sahani</t>
         </is>
       </c>
-      <c r="O14" s="2" t="inlineStr">
-        <is>
-          <t>9869745682</t>
-        </is>
+      <c r="O14" s="2" t="n">
+        <v>9869745682</v>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
@@ -3735,10 +3987,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y14" s="2" t="inlineStr">
-        <is>
-          <t>27.69665</t>
-        </is>
+      <c r="Y14" s="2" t="n">
+        <v>27.69665</v>
       </c>
       <c r="Z14" s="2" t="inlineStr">
         <is>
@@ -3794,20 +4044,16 @@
           <t>Sabin Giri</t>
         </is>
       </c>
-      <c r="AN14" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN14" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO14" s="2" t="inlineStr">
         <is>
           <t>L3-2</t>
         </is>
       </c>
-      <c r="AP14" s="2" t="inlineStr">
-        <is>
-          <t>85.33558</t>
-        </is>
+      <c r="AP14" s="2" t="n">
+        <v>85.33557999999999</v>
       </c>
       <c r="AQ14" s="2" t="inlineStr"/>
       <c r="AR14" s="2" t="inlineStr">
@@ -3844,6 +4090,9 @@
         <is>
           <t>Sabin Giri</t>
         </is>
+      </c>
+      <c r="AY14" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -3913,10 +4162,8 @@
           <t>Shankar Sharma</t>
         </is>
       </c>
-      <c r="O15" s="2" t="inlineStr">
-        <is>
-          <t>9857631208</t>
-        </is>
+      <c r="O15" s="2" t="n">
+        <v>9857631208</v>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
@@ -3951,10 +4198,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y15" s="2" t="inlineStr">
-        <is>
-          <t>27.69312</t>
-        </is>
+      <c r="Y15" s="2" t="n">
+        <v>27.69312</v>
       </c>
       <c r="Z15" s="2" t="inlineStr">
         <is>
@@ -4010,20 +4255,16 @@
           <t>Binod Dhami</t>
         </is>
       </c>
-      <c r="AN15" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN15" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO15" s="2" t="inlineStr">
         <is>
           <t>L46-4</t>
         </is>
       </c>
-      <c r="AP15" s="2" t="inlineStr">
-        <is>
-          <t>85.33458</t>
-        </is>
+      <c r="AP15" s="2" t="n">
+        <v>85.33458</v>
       </c>
       <c r="AQ15" s="2" t="inlineStr"/>
       <c r="AR15" s="2" t="inlineStr">
@@ -4060,6 +4301,9 @@
         <is>
           <t>Sabin Giri</t>
         </is>
+      </c>
+      <c r="AY15" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -4129,10 +4373,8 @@
           <t>Sujan Adhikari</t>
         </is>
       </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>9846523247</t>
-        </is>
+      <c r="O16" s="2" t="n">
+        <v>9846523247</v>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
@@ -4167,10 +4409,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y16" s="2" t="inlineStr">
-        <is>
-          <t>27.74276</t>
-        </is>
+      <c r="Y16" s="2" t="n">
+        <v>27.74276</v>
       </c>
       <c r="Z16" s="2" t="inlineStr">
         <is>
@@ -4208,10 +4448,8 @@
           <t>Router Upgrade  Wi-Fi 6</t>
         </is>
       </c>
-      <c r="AH16" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="AH16" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="AI16" s="2" t="inlineStr">
         <is>
@@ -4230,20 +4468,16 @@
           <t>Sanjeev Giri</t>
         </is>
       </c>
-      <c r="AN16" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="AN16" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="AO16" s="2" t="inlineStr">
         <is>
           <t>1,14</t>
         </is>
       </c>
-      <c r="AP16" s="2" t="inlineStr">
-        <is>
-          <t>85.32963</t>
-        </is>
+      <c r="AP16" s="2" t="n">
+        <v>85.32962999999999</v>
       </c>
       <c r="AQ16" s="2" t="inlineStr"/>
       <c r="AR16" s="2" t="inlineStr">
@@ -4280,6 +4514,9 @@
         <is>
           <t>Sanjeev Giri</t>
         </is>
+      </c>
+      <c r="AY16" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -4349,10 +4586,8 @@
           <t>Shyam Maharjan</t>
         </is>
       </c>
-      <c r="O17" s="2" t="inlineStr">
-        <is>
-          <t>9841390761</t>
-        </is>
+      <c r="O17" s="2" t="n">
+        <v>9841390761</v>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
@@ -4442,10 +4677,8 @@
           <t>Sanjeev Giri</t>
         </is>
       </c>
-      <c r="AN17" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="AN17" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="AO17" s="2" t="inlineStr">
         <is>
@@ -4489,6 +4722,9 @@
           <t>Sanjeev Giri</t>
         </is>
       </c>
+      <c r="AY17" s="2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -4557,10 +4793,8 @@
           <t>Shyam Maharjan</t>
         </is>
       </c>
-      <c r="O18" s="2" t="inlineStr">
-        <is>
-          <t>9841390761</t>
-        </is>
+      <c r="O18" s="2" t="n">
+        <v>9841390761</v>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
@@ -4650,10 +4884,8 @@
           <t>Sanjeev Giri</t>
         </is>
       </c>
-      <c r="AN18" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="AN18" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="AO18" s="2" t="inlineStr">
         <is>
@@ -4697,6 +4929,9 @@
           <t>Sanjeev Giri</t>
         </is>
       </c>
+      <c r="AY18" s="2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -4765,10 +5000,8 @@
           <t>Sandesh Mudbhari</t>
         </is>
       </c>
-      <c r="O19" s="2" t="inlineStr">
-        <is>
-          <t>9761303470</t>
-        </is>
+      <c r="O19" s="2" t="n">
+        <v>9761303470</v>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
@@ -4803,10 +5036,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y19" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="Y19" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="Z19" s="2" t="inlineStr">
         <is>
@@ -4862,20 +5093,16 @@
           <t>Sanjeev Giri</t>
         </is>
       </c>
-      <c r="AN19" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="AN19" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="AO19" s="2" t="inlineStr">
         <is>
           <t>1,11</t>
         </is>
       </c>
-      <c r="AP19" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="AP19" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="AQ19" s="2" t="inlineStr"/>
       <c r="AR19" s="2" t="inlineStr">
@@ -4912,6 +5139,9 @@
         <is>
           <t>Sanjeev Giri</t>
         </is>
+      </c>
+      <c r="AY19" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -4981,10 +5211,8 @@
           <t>Badri Bikram kafle</t>
         </is>
       </c>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>9844197691</t>
-        </is>
+      <c r="O20" s="2" t="n">
+        <v>9844197691</v>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
@@ -5074,10 +5302,8 @@
           <t>Sanjeev Giri</t>
         </is>
       </c>
-      <c r="AN20" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="AN20" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="AO20" s="2" t="inlineStr">
         <is>
@@ -5121,6 +5347,9 @@
           <t>Sanjeev Giri</t>
         </is>
       </c>
+      <c r="AY20" s="2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -5189,10 +5418,8 @@
           <t>Man Bahadur Gurung</t>
         </is>
       </c>
-      <c r="O21" s="2" t="inlineStr">
-        <is>
-          <t>9864627161</t>
-        </is>
+      <c r="O21" s="2" t="n">
+        <v>9864627161</v>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
@@ -5227,10 +5454,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y21" s="2" t="inlineStr">
-        <is>
-          <t>27.720112</t>
-        </is>
+      <c r="Y21" s="2" t="n">
+        <v>27.720112</v>
       </c>
       <c r="Z21" s="2" t="inlineStr">
         <is>
@@ -5282,20 +5507,16 @@
           <t>Binod Dhami</t>
         </is>
       </c>
-      <c r="AN21" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="AN21" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="AO21" s="2" t="inlineStr">
         <is>
           <t>4,3</t>
         </is>
       </c>
-      <c r="AP21" s="2" t="inlineStr">
-        <is>
-          <t>85.311673</t>
-        </is>
+      <c r="AP21" s="2" t="n">
+        <v>85.311673</v>
       </c>
       <c r="AQ21" s="2" t="inlineStr"/>
       <c r="AR21" s="2" t="inlineStr">
@@ -5332,6 +5553,9 @@
         <is>
           <t>Sanjeev Giri</t>
         </is>
+      </c>
+      <c r="AY21" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -5401,10 +5625,8 @@
           <t>Jay Prakash Chaudhary</t>
         </is>
       </c>
-      <c r="O22" s="2" t="inlineStr">
-        <is>
-          <t>9808528372</t>
-        </is>
+      <c r="O22" s="2" t="n">
+        <v>9808528372</v>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
@@ -5439,10 +5661,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y22" s="2" t="inlineStr">
-        <is>
-          <t>27.729885</t>
-        </is>
+      <c r="Y22" s="2" t="n">
+        <v>27.729885</v>
       </c>
       <c r="Z22" s="2" t="inlineStr">
         <is>
@@ -5494,20 +5714,16 @@
           <t>Binod Dhami</t>
         </is>
       </c>
-      <c r="AN22" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN22" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO22" s="2" t="inlineStr">
         <is>
           <t>L33-1</t>
         </is>
       </c>
-      <c r="AP22" s="2" t="inlineStr">
-        <is>
-          <t>85.312287</t>
-        </is>
+      <c r="AP22" s="2" t="n">
+        <v>85.312287</v>
       </c>
       <c r="AQ22" s="2" t="inlineStr"/>
       <c r="AR22" s="2" t="inlineStr">
@@ -5544,6 +5760,9 @@
         <is>
           <t>Sanjeev Giri</t>
         </is>
+      </c>
+      <c r="AY22" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -5613,10 +5832,8 @@
           <t>Rojan Bajracharya</t>
         </is>
       </c>
-      <c r="O23" s="2" t="inlineStr">
-        <is>
-          <t>9860350871</t>
-        </is>
+      <c r="O23" s="2" t="n">
+        <v>9860350871</v>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
@@ -5651,10 +5868,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y23" s="2" t="inlineStr">
-        <is>
-          <t>27.67455</t>
-        </is>
+      <c r="Y23" s="2" t="n">
+        <v>27.67455</v>
       </c>
       <c r="Z23" s="2" t="inlineStr">
         <is>
@@ -5710,20 +5925,16 @@
           <t>Chandramani Tharu</t>
         </is>
       </c>
-      <c r="AN23" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN23" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO23" s="2" t="inlineStr">
         <is>
           <t>L41-1</t>
         </is>
       </c>
-      <c r="AP23" s="2" t="inlineStr">
-        <is>
-          <t>85.32104</t>
-        </is>
+      <c r="AP23" s="2" t="n">
+        <v>85.32104</v>
       </c>
       <c r="AQ23" s="2" t="inlineStr"/>
       <c r="AR23" s="2" t="inlineStr">
@@ -5760,6 +5971,9 @@
         <is>
           <t>Chandramani Tharu</t>
         </is>
+      </c>
+      <c r="AY23" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -5829,10 +6043,8 @@
           <t>Rojan Bajracharya</t>
         </is>
       </c>
-      <c r="O24" s="2" t="inlineStr">
-        <is>
-          <t>9860350871</t>
-        </is>
+      <c r="O24" s="2" t="n">
+        <v>9860350871</v>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
@@ -5867,10 +6079,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y24" s="2" t="inlineStr">
-        <is>
-          <t>27.67455</t>
-        </is>
+      <c r="Y24" s="2" t="n">
+        <v>27.67455</v>
       </c>
       <c r="Z24" s="2" t="inlineStr">
         <is>
@@ -5926,20 +6136,16 @@
           <t>Chandramani Tharu</t>
         </is>
       </c>
-      <c r="AN24" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN24" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO24" s="2" t="inlineStr">
         <is>
           <t>L41-1</t>
         </is>
       </c>
-      <c r="AP24" s="2" t="inlineStr">
-        <is>
-          <t>85.32104</t>
-        </is>
+      <c r="AP24" s="2" t="n">
+        <v>85.32104</v>
       </c>
       <c r="AQ24" s="2" t="inlineStr"/>
       <c r="AR24" s="2" t="inlineStr">
@@ -5976,6 +6182,9 @@
         <is>
           <t>Chandramani Tharu</t>
         </is>
+      </c>
+      <c r="AY24" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -6045,10 +6254,8 @@
           <t>chitra kumar subedi</t>
         </is>
       </c>
-      <c r="O25" s="2" t="inlineStr">
-        <is>
-          <t>9841982586</t>
-        </is>
+      <c r="O25" s="2" t="n">
+        <v>9841982586</v>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
@@ -6083,10 +6290,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y25" s="2" t="inlineStr">
-        <is>
-          <t>27.70074</t>
-        </is>
+      <c r="Y25" s="2" t="n">
+        <v>27.70074</v>
       </c>
       <c r="Z25" s="2" t="inlineStr">
         <is>
@@ -6142,20 +6347,16 @@
           <t>Chandramani Tharu</t>
         </is>
       </c>
-      <c r="AN25" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN25" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO25" s="2" t="inlineStr">
         <is>
           <t>L48-3</t>
         </is>
       </c>
-      <c r="AP25" s="2" t="inlineStr">
-        <is>
-          <t>85.34949</t>
-        </is>
+      <c r="AP25" s="2" t="n">
+        <v>85.34949</v>
       </c>
       <c r="AQ25" s="2" t="inlineStr"/>
       <c r="AR25" s="2" t="inlineStr">
@@ -6192,6 +6393,9 @@
         <is>
           <t>Chandramani Tharu</t>
         </is>
+      </c>
+      <c r="AY25" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -6261,10 +6465,8 @@
           <t>Saugat Lawfirm</t>
         </is>
       </c>
-      <c r="O26" s="2" t="inlineStr">
-        <is>
-          <t>9841255369</t>
-        </is>
+      <c r="O26" s="2" t="n">
+        <v>9841255369</v>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
@@ -6299,10 +6501,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y26" s="2" t="inlineStr">
-        <is>
-          <t>27.689155</t>
-        </is>
+      <c r="Y26" s="2" t="n">
+        <v>27.689155</v>
       </c>
       <c r="Z26" s="2" t="inlineStr">
         <is>
@@ -6358,20 +6558,16 @@
           <t>Chandramani Tharu</t>
         </is>
       </c>
-      <c r="AN26" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="AN26" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="AO26" s="2" t="inlineStr">
         <is>
           <t>3,2</t>
         </is>
       </c>
-      <c r="AP26" s="2" t="inlineStr">
-        <is>
-          <t>85.324218</t>
-        </is>
+      <c r="AP26" s="2" t="n">
+        <v>85.324218</v>
       </c>
       <c r="AQ26" s="2" t="inlineStr"/>
       <c r="AR26" s="2" t="inlineStr">
@@ -6408,6 +6604,9 @@
         <is>
           <t>Chandramani Tharu</t>
         </is>
+      </c>
+      <c r="AY26" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -6477,10 +6676,8 @@
           <t>Kanunalaya Inc. Pvt Ltd</t>
         </is>
       </c>
-      <c r="O27" s="2" t="inlineStr">
-        <is>
-          <t>9851177792</t>
-        </is>
+      <c r="O27" s="2" t="n">
+        <v>9851177792</v>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
@@ -6515,10 +6712,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y27" s="2" t="inlineStr">
-        <is>
-          <t>27.69393</t>
-        </is>
+      <c r="Y27" s="2" t="n">
+        <v>27.69393</v>
       </c>
       <c r="Z27" s="2" t="inlineStr">
         <is>
@@ -6570,20 +6765,16 @@
           <t>Chandramani Tharu</t>
         </is>
       </c>
-      <c r="AN27" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN27" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO27" s="2" t="inlineStr">
         <is>
           <t>L47-2</t>
         </is>
       </c>
-      <c r="AP27" s="2" t="inlineStr">
-        <is>
-          <t>85.331616</t>
-        </is>
+      <c r="AP27" s="2" t="n">
+        <v>85.331616</v>
       </c>
       <c r="AQ27" s="2" t="inlineStr"/>
       <c r="AR27" s="2" t="inlineStr">
@@ -6620,6 +6811,9 @@
         <is>
           <t>Chandramani Tharu</t>
         </is>
+      </c>
+      <c r="AY27" s="2" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -6689,10 +6883,8 @@
           <t>Habib Laheri</t>
         </is>
       </c>
-      <c r="O28" s="2" t="inlineStr">
-        <is>
-          <t>9851029384</t>
-        </is>
+      <c r="O28" s="2" t="n">
+        <v>9851029384</v>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
@@ -6727,10 +6919,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y28" s="2" t="inlineStr">
-        <is>
-          <t>27.70816</t>
-        </is>
+      <c r="Y28" s="2" t="n">
+        <v>27.70816</v>
       </c>
       <c r="Z28" s="2" t="inlineStr">
         <is>
@@ -6782,20 +6972,16 @@
           <t>Chandramani Tharu</t>
         </is>
       </c>
-      <c r="AN28" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="AN28" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="AO28" s="2" t="inlineStr">
         <is>
           <t>3,13</t>
         </is>
       </c>
-      <c r="AP28" s="2" t="inlineStr">
-        <is>
-          <t>85.31304</t>
-        </is>
+      <c r="AP28" s="2" t="n">
+        <v>85.31304</v>
       </c>
       <c r="AQ28" s="2" t="inlineStr"/>
       <c r="AR28" s="2" t="inlineStr">
@@ -6832,6 +7018,9 @@
         <is>
           <t>Chandramani Tharu</t>
         </is>
+      </c>
+      <c r="AY28" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -6901,10 +7090,8 @@
           <t>Rakesh Shrestha</t>
         </is>
       </c>
-      <c r="O29" s="2" t="inlineStr">
-        <is>
-          <t>9861209491</t>
-        </is>
+      <c r="O29" s="2" t="n">
+        <v>9861209491</v>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
@@ -6939,10 +7126,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y29" s="2" t="inlineStr">
-        <is>
-          <t>27.71045</t>
-        </is>
+      <c r="Y29" s="2" t="n">
+        <v>27.71045</v>
       </c>
       <c r="Z29" s="2" t="inlineStr">
         <is>
@@ -6994,20 +7179,16 @@
           <t>Binod Dhami</t>
         </is>
       </c>
-      <c r="AN29" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="AN29" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="AO29" s="2" t="inlineStr">
         <is>
           <t>2,10</t>
         </is>
       </c>
-      <c r="AP29" s="2" t="inlineStr">
-        <is>
-          <t>85.299958</t>
-        </is>
+      <c r="AP29" s="2" t="n">
+        <v>85.299958</v>
       </c>
       <c r="AQ29" s="2" t="inlineStr"/>
       <c r="AR29" s="2" t="inlineStr">
@@ -7044,6 +7225,9 @@
         <is>
           <t>Chandramani Tharu</t>
         </is>
+      </c>
+      <c r="AY29" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -7113,10 +7297,8 @@
           <t>Sanjeev Rijal</t>
         </is>
       </c>
-      <c r="O30" s="2" t="inlineStr">
-        <is>
-          <t>9860676817</t>
-        </is>
+      <c r="O30" s="2" t="n">
+        <v>9860676817</v>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
@@ -7151,10 +7333,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y30" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="Y30" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="Z30" s="2" t="inlineStr">
         <is>
@@ -7210,20 +7390,16 @@
           <t>Sunil Chaudhary</t>
         </is>
       </c>
-      <c r="AN30" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN30" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO30" s="2" t="inlineStr">
         <is>
           <t>CDB278</t>
         </is>
       </c>
-      <c r="AP30" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="AP30" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="AQ30" s="2" t="inlineStr"/>
       <c r="AR30" s="2" t="inlineStr">
@@ -7260,6 +7436,9 @@
         <is>
           <t>Sunil Chaudhary</t>
         </is>
+      </c>
+      <c r="AY30" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -7329,10 +7508,8 @@
           <t>Sanjeev Rijal</t>
         </is>
       </c>
-      <c r="O31" s="2" t="inlineStr">
-        <is>
-          <t>9860676817</t>
-        </is>
+      <c r="O31" s="2" t="n">
+        <v>9860676817</v>
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
@@ -7367,10 +7544,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y31" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="Y31" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="Z31" s="2" t="inlineStr">
         <is>
@@ -7426,20 +7601,16 @@
           <t>Sunil Chaudhary</t>
         </is>
       </c>
-      <c r="AN31" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN31" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO31" s="2" t="inlineStr">
         <is>
           <t>CDB278</t>
         </is>
       </c>
-      <c r="AP31" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="AP31" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="AQ31" s="2" t="inlineStr"/>
       <c r="AR31" s="2" t="inlineStr">
@@ -7476,6 +7647,9 @@
         <is>
           <t>Sunil Chaudhary</t>
         </is>
+      </c>
+      <c r="AY31" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -7545,10 +7719,8 @@
           <t>Uma Sankar Prasad</t>
         </is>
       </c>
-      <c r="O32" s="2" t="inlineStr">
-        <is>
-          <t>9851216612</t>
-        </is>
+      <c r="O32" s="2" t="n">
+        <v>9851216612</v>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
@@ -7583,10 +7755,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y32" s="2" t="inlineStr">
-        <is>
-          <t>27.71082</t>
-        </is>
+      <c r="Y32" s="2" t="n">
+        <v>27.71082</v>
       </c>
       <c r="Z32" s="2" t="inlineStr">
         <is>
@@ -7642,20 +7812,16 @@
           <t>Sunil Chaudhary</t>
         </is>
       </c>
-      <c r="AN32" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="AN32" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="AO32" s="2" t="inlineStr">
         <is>
           <t>3,13</t>
         </is>
       </c>
-      <c r="AP32" s="2" t="inlineStr">
-        <is>
-          <t>85.28612</t>
-        </is>
+      <c r="AP32" s="2" t="n">
+        <v>85.28612</v>
       </c>
       <c r="AQ32" s="2" t="inlineStr"/>
       <c r="AR32" s="2" t="inlineStr">
@@ -7692,6 +7858,9 @@
         <is>
           <t>Sunil Chaudhary</t>
         </is>
+      </c>
+      <c r="AY32" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -7761,10 +7930,8 @@
           <t>Uma Sankar Prasad</t>
         </is>
       </c>
-      <c r="O33" s="2" t="inlineStr">
-        <is>
-          <t>9851216612</t>
-        </is>
+      <c r="O33" s="2" t="n">
+        <v>9851216612</v>
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
@@ -7799,10 +7966,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y33" s="2" t="inlineStr">
-        <is>
-          <t>27.71082</t>
-        </is>
+      <c r="Y33" s="2" t="n">
+        <v>27.71082</v>
       </c>
       <c r="Z33" s="2" t="inlineStr">
         <is>
@@ -7858,20 +8023,16 @@
           <t>Sunil Chaudhary</t>
         </is>
       </c>
-      <c r="AN33" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="AN33" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="AO33" s="2" t="inlineStr">
         <is>
           <t>3,13</t>
         </is>
       </c>
-      <c r="AP33" s="2" t="inlineStr">
-        <is>
-          <t>85.28612</t>
-        </is>
+      <c r="AP33" s="2" t="n">
+        <v>85.28612</v>
       </c>
       <c r="AQ33" s="2" t="inlineStr"/>
       <c r="AR33" s="2" t="inlineStr">
@@ -7908,6 +8069,9 @@
         <is>
           <t>Sunil Chaudhary</t>
         </is>
+      </c>
+      <c r="AY33" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -7977,10 +8141,8 @@
           <t>Humesh Ratna Tuladhar</t>
         </is>
       </c>
-      <c r="O34" s="2" t="inlineStr">
-        <is>
-          <t>9847473679</t>
-        </is>
+      <c r="O34" s="2" t="n">
+        <v>9847473679</v>
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
@@ -8066,10 +8228,8 @@
           <t>Sunil Chaudhary</t>
         </is>
       </c>
-      <c r="AN34" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="AN34" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="AO34" s="2" t="inlineStr">
         <is>
@@ -8113,6 +8273,9 @@
           <t>Sunil Chaudhary</t>
         </is>
       </c>
+      <c r="AY34" s="2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -8181,10 +8344,8 @@
           <t>Humesh Ratna Tuladhar</t>
         </is>
       </c>
-      <c r="O35" s="2" t="inlineStr">
-        <is>
-          <t>9847473679</t>
-        </is>
+      <c r="O35" s="2" t="n">
+        <v>9847473679</v>
       </c>
       <c r="P35" s="2" t="inlineStr">
         <is>
@@ -8270,10 +8431,8 @@
           <t>Sunil Chaudhary</t>
         </is>
       </c>
-      <c r="AN35" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="AN35" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="AO35" s="2" t="inlineStr">
         <is>
@@ -8317,6 +8476,9 @@
           <t>Sunil Chaudhary</t>
         </is>
       </c>
+      <c r="AY35" s="2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -8385,10 +8547,8 @@
           <t>Amit Thakur</t>
         </is>
       </c>
-      <c r="O36" s="2" t="inlineStr">
-        <is>
-          <t>9849459569</t>
-        </is>
+      <c r="O36" s="2" t="n">
+        <v>9849459569</v>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
@@ -8423,10 +8583,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y36" s="2" t="inlineStr">
-        <is>
-          <t>27.70339</t>
-        </is>
+      <c r="Y36" s="2" t="n">
+        <v>27.70339</v>
       </c>
       <c r="Z36" s="2" t="inlineStr">
         <is>
@@ -8482,20 +8640,16 @@
           <t>Sunil Chaudhary</t>
         </is>
       </c>
-      <c r="AN36" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN36" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO36" s="2" t="inlineStr">
         <is>
           <t>CDB117</t>
         </is>
       </c>
-      <c r="AP36" s="2" t="inlineStr">
-        <is>
-          <t>85.2894</t>
-        </is>
+      <c r="AP36" s="2" t="n">
+        <v>85.2894</v>
       </c>
       <c r="AQ36" s="2" t="inlineStr"/>
       <c r="AR36" s="2" t="inlineStr">
@@ -8532,6 +8686,9 @@
         <is>
           <t>Sunil Chaudhary</t>
         </is>
+      </c>
+      <c r="AY36" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -8601,10 +8758,8 @@
           <t>Prashansa Lamichhane</t>
         </is>
       </c>
-      <c r="O37" s="2" t="inlineStr">
-        <is>
-          <t>9843467444</t>
-        </is>
+      <c r="O37" s="2" t="n">
+        <v>9843467444</v>
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
@@ -8639,10 +8794,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y37" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="Y37" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="Z37" s="2" t="inlineStr">
         <is>
@@ -8694,20 +8847,16 @@
           <t>Sunil Chaudhary</t>
         </is>
       </c>
-      <c r="AN37" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN37" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO37" s="2" t="inlineStr">
         <is>
           <t>CDB058</t>
         </is>
       </c>
-      <c r="AP37" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="AP37" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="AQ37" s="2" t="inlineStr"/>
       <c r="AR37" s="2" t="inlineStr">
@@ -8744,6 +8893,9 @@
         <is>
           <t>Sunil Chaudhary</t>
         </is>
+      </c>
+      <c r="AY37" s="2" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -8813,10 +8965,8 @@
           <t>Prashansa Lamichhane</t>
         </is>
       </c>
-      <c r="O38" s="2" t="inlineStr">
-        <is>
-          <t>9843467444</t>
-        </is>
+      <c r="O38" s="2" t="n">
+        <v>9843467444</v>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
@@ -8851,10 +9001,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y38" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="Y38" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="Z38" s="2" t="inlineStr">
         <is>
@@ -8906,20 +9054,16 @@
           <t>Sunil Chaudhary</t>
         </is>
       </c>
-      <c r="AN38" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN38" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO38" s="2" t="inlineStr">
         <is>
           <t>CDB058</t>
         </is>
       </c>
-      <c r="AP38" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="AP38" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="AQ38" s="2" t="inlineStr"/>
       <c r="AR38" s="2" t="inlineStr">
@@ -8956,6 +9100,9 @@
         <is>
           <t>Sunil Chaudhary</t>
         </is>
+      </c>
+      <c r="AY38" s="2" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -9025,10 +9172,8 @@
           <t>Mala Rai</t>
         </is>
       </c>
-      <c r="O39" s="2" t="inlineStr">
-        <is>
-          <t>9841922058</t>
-        </is>
+      <c r="O39" s="2" t="n">
+        <v>9841922058</v>
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
@@ -9118,10 +9263,8 @@
           <t>Sunil Chaudhary</t>
         </is>
       </c>
-      <c r="AN39" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="AN39" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="AO39" s="2" t="inlineStr">
         <is>
@@ -9165,6 +9308,9 @@
           <t>Sunil Chaudhary</t>
         </is>
       </c>
+      <c r="AY39" s="2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -9233,10 +9379,8 @@
           <t>Babu krishna maharjan</t>
         </is>
       </c>
-      <c r="O40" s="2" t="inlineStr">
-        <is>
-          <t>9702036701</t>
-        </is>
+      <c r="O40" s="2" t="n">
+        <v>9702036701</v>
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
@@ -9326,10 +9470,8 @@
           <t>Sunil Chaudhary</t>
         </is>
       </c>
-      <c r="AN40" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="AN40" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="AO40" s="2" t="inlineStr">
         <is>
@@ -9373,6 +9515,9 @@
           <t>Sunil Chaudhary</t>
         </is>
       </c>
+      <c r="AY40" s="2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -9441,10 +9586,8 @@
           <t>Babu krishna maharjan</t>
         </is>
       </c>
-      <c r="O41" s="2" t="inlineStr">
-        <is>
-          <t>9702036701</t>
-        </is>
+      <c r="O41" s="2" t="n">
+        <v>9702036701</v>
       </c>
       <c r="P41" s="2" t="inlineStr">
         <is>
@@ -9534,10 +9677,8 @@
           <t>Sunil Chaudhary</t>
         </is>
       </c>
-      <c r="AN41" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="AN41" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="AO41" s="2" t="inlineStr">
         <is>
@@ -9581,6 +9722,9 @@
           <t>Sunil Chaudhary</t>
         </is>
       </c>
+      <c r="AY41" s="2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -9649,10 +9793,8 @@
           <t>sigma refrigeration</t>
         </is>
       </c>
-      <c r="O42" s="2" t="inlineStr">
-        <is>
-          <t>9813064680</t>
-        </is>
+      <c r="O42" s="2" t="n">
+        <v>9813064680</v>
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
@@ -9742,10 +9884,8 @@
           <t>Binod Dhami</t>
         </is>
       </c>
-      <c r="AN42" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN42" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO42" s="2" t="inlineStr">
         <is>
@@ -9789,6 +9929,9 @@
           <t>Sunil Chaudhary</t>
         </is>
       </c>
+      <c r="AY42" s="2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -9857,10 +10000,8 @@
           <t>sigma refrigeration</t>
         </is>
       </c>
-      <c r="O43" s="2" t="inlineStr">
-        <is>
-          <t>9813064680</t>
-        </is>
+      <c r="O43" s="2" t="n">
+        <v>9813064680</v>
       </c>
       <c r="P43" s="2" t="inlineStr">
         <is>
@@ -9950,10 +10091,8 @@
           <t>Binod Dhami</t>
         </is>
       </c>
-      <c r="AN43" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN43" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO43" s="2" t="inlineStr">
         <is>
@@ -9997,6 +10136,9 @@
           <t>Sunil Chaudhary</t>
         </is>
       </c>
+      <c r="AY43" s="2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -10065,10 +10207,8 @@
           <t>Anupama  Thapa</t>
         </is>
       </c>
-      <c r="O44" s="2" t="inlineStr">
-        <is>
-          <t>9857030718</t>
-        </is>
+      <c r="O44" s="2" t="n">
+        <v>9857030718</v>
       </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
@@ -10158,10 +10298,8 @@
           <t>Sunil Chaudhary</t>
         </is>
       </c>
-      <c r="AN44" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN44" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO44" s="2" t="inlineStr">
         <is>
@@ -10205,6 +10343,9 @@
           <t>Sunil Chaudhary</t>
         </is>
       </c>
+      <c r="AY44" s="2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -10273,10 +10414,8 @@
           <t>Anupama  Thapa</t>
         </is>
       </c>
-      <c r="O45" s="2" t="inlineStr">
-        <is>
-          <t>9857030718</t>
-        </is>
+      <c r="O45" s="2" t="n">
+        <v>9857030718</v>
       </c>
       <c r="P45" s="2" t="inlineStr">
         <is>
@@ -10366,10 +10505,8 @@
           <t>Sunil Chaudhary</t>
         </is>
       </c>
-      <c r="AN45" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN45" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO45" s="2" t="inlineStr">
         <is>
@@ -10412,6 +10549,9 @@
         <is>
           <t>Sunil Chaudhary</t>
         </is>
+      </c>
+      <c r="AY45" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix Grand Total column position to far right and add deduplication to prevent double-counting
</commit_message>
<xml_diff>
--- a/EXECUTIVE_TEAM_AUDIT_REPORT_14_Sep_2026.xlsx
+++ b/EXECUTIVE_TEAM_AUDIT_REPORT_14_Sep_2026.xlsx
@@ -823,7 +823,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>3</v>
@@ -832,22 +832,22 @@
         <v>4</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>4</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>37</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Router Adaptor damage Issue</t>
+          <t>NETTV-Channel buffering,feeze issue</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
@@ -857,7 +857,7 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>0</v>
@@ -866,10 +866,10 @@
         <v>0</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -903,7 +903,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>NETTV-Channel buffering,feeze issue</t>
+          <t>Router Adaptor damage Issue</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
@@ -913,7 +913,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0</v>
@@ -922,7 +922,7 @@
         <v>0</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5" s="4" t="n">
         <v>1</v>
@@ -1019,7 +1019,7 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C9" s="3" t="n">
         <v>3</v>
@@ -1028,16 +1028,16 @@
         <v>6</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>5</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>44</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>